<commit_message>
Version 9: Add data upload workflow and revision log
</commit_message>
<xml_diff>
--- a/outputs/cbs_somalia_macro_model_outputs.xlsx
+++ b/outputs/cbs_somalia_macro_model_outputs.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Key_Indicators" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Macro_Framework" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Real_Sector" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="External_Sector" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Fiscal_Sector" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Monetary_Sector" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GDP_Reconciliation" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Nominal_GDP_Output" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Data_Checks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Indicators" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Macro_Framework" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Real_Sector" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External_Sector" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal_Sector" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monetary_Sector" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GDP_Reconciliation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nominal_GDP_Output" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Checks" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR13"/>
+  <dimension ref="A1:AW13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,6 +576,21 @@
       <c r="AR1" s="1" t="n">
         <v>2030</v>
       </c>
+      <c r="AS1" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="AT1" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="AU1" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="AV1" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="AW1" s="1" t="n">
+        <v>2035</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -716,6 +731,21 @@
       <c r="AR2" t="n">
         <v>19060.63907040565</v>
       </c>
+      <c r="AS2" t="n">
+        <v>20598.21018872874</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>22259.81308453677</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>24055.45307182318</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>25995.94256668169</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>28092.96619408858</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -856,6 +886,21 @@
       <c r="AR3" t="n">
         <v>11025.6946566189</v>
       </c>
+      <c r="AS3" t="n">
+        <v>11430.14830089831</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>11849.43844804356</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>12284.10934291535</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>12734.72519481419</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>13201.87090983246</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -996,6 +1041,21 @@
       <c r="AR4" t="n">
         <v>32336.22363849695</v>
       </c>
+      <c r="AS4" t="n">
+        <v>36032.19101047174</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>40150.60025696988</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>44739.73566215356</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>49853.4003099469</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>55551.5468721194</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1136,6 +1196,21 @@
       <c r="AR5" t="n">
         <v>11724.79872189115</v>
       </c>
+      <c r="AS5" t="n">
+        <v>14557.1162302894</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>18073.62650469237</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>22439.60753376663</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>27860.26291617487</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>34590.36654675839</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1275,6 +1350,21 @@
       </c>
       <c r="AR6" t="n">
         <v>-0.5102954804154141</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>-0.7090768402309638</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>-0.9642492908551845</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>-1.290998032100474</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>-1.70832487995135</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>-2.239975698570109</v>
       </c>
     </row>
     <row r="7">
@@ -1346,6 +1436,21 @@
       <c r="AR7" t="n">
         <v>1632.434921638175</v>
       </c>
+      <c r="AS7" t="n">
+        <v>1801.109543185191</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>1988.776833185599</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>2197.764223574542</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>2430.70562780798</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>2690.584037991505</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1416,6 +1521,21 @@
       <c r="AR8" t="n">
         <v>1069.338020086677</v>
       </c>
+      <c r="AS8" t="n">
+        <v>1155.598677420192</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>1248.817752825298</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>1349.556563402464</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>1458.421706211489</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>1576.068710885532</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1486,6 +1606,21 @@
       <c r="AR9" t="n">
         <v>0.0295423935929717</v>
       </c>
+      <c r="AS9" t="n">
+        <v>0.03133820171027384</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.03324192694476528</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>0.03526051484624112</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.03740137212191884</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.03967239768866034</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1556,6 +1691,21 @@
       <c r="AR10" t="n">
         <v>0</v>
       </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1639,6 +1789,21 @@
       </c>
       <c r="AR11" t="n">
         <v>-0.04263048365570885</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0.3376025344932318</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0.9823609317833634</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>2.054282991927361</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>3.819131097471031</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>6.712985895676991</v>
       </c>
     </row>
     <row r="12">
@@ -1710,6 +1875,21 @@
       <c r="AR12" t="n">
         <v>0.1282302625475281</v>
       </c>
+      <c r="AS12" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>0.1282302625475281</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1780,6 +1960,21 @@
       <c r="AR13" t="n">
         <v>0.03488961903310435</v>
       </c>
+      <c r="AS13" t="n">
+        <v>0.03488961903310435</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0.03488961903310435</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1903,7 +2098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR49"/>
+  <dimension ref="A1:AW49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2045,6 +2240,21 @@
       <c r="AR1" s="1" t="n">
         <v>2030</v>
       </c>
+      <c r="AS1" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="AT1" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="AU1" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="AV1" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="AW1" s="1" t="n">
+        <v>2035</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2185,6 +2395,21 @@
       <c r="AR2" t="n">
         <v>19060.63907040565</v>
       </c>
+      <c r="AS2" t="n">
+        <v>20598.21018872874</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>22259.81308453677</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>24055.45307182318</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>25995.94256668169</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>28092.96619408858</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2325,6 +2550,21 @@
       <c r="AR3" t="n">
         <v>11025.6946566189</v>
       </c>
+      <c r="AS3" t="n">
+        <v>11430.14830089831</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>11849.43844804356</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>12284.10934291535</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>12734.72519481419</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>13201.87090983246</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2465,6 +2705,21 @@
       <c r="AR4" t="n">
         <v>32336.22363849695</v>
       </c>
+      <c r="AS4" t="n">
+        <v>36032.19101047174</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>40150.60025696988</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>44739.73566215356</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>49853.4003099469</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>55551.5468721194</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2605,6 +2860,21 @@
       <c r="AR5" t="n">
         <v>30553.60246145808</v>
       </c>
+      <c r="AS5" t="n">
+        <v>34045.74259536669</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>37937.01873067608</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>42273.05032751824</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>47104.6709463204</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>52488.52419615267</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2745,6 +3015,21 @@
       <c r="AR6" t="n">
         <v>1782.621177038872</v>
       </c>
+      <c r="AS6" t="n">
+        <v>1986.448415105047</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>2213.581526293798</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>2466.685334635314</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>2748.729363626501</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>3063.02267596673</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2885,6 +3170,21 @@
       <c r="AR7" t="n">
         <v>11724.79872189115</v>
       </c>
+      <c r="AS7" t="n">
+        <v>14557.1162302894</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>18073.62650469237</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>22439.60753376663</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>27860.26291617487</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>34590.36654675839</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3025,6 +3325,21 @@
       <c r="AR8" t="n">
         <v>25369.9732236226</v>
       </c>
+      <c r="AS8" t="n">
+        <v>33826.20841313917</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>45104.07584846929</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>60146.11618048123</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>80210.06936750493</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>106974.4018076055</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3165,6 +3480,21 @@
       <c r="AR9" t="n">
         <v>40643.7985421476</v>
       </c>
+      <c r="AS9" t="n">
+        <v>49211.59167013455</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>59604.48054426122</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>72214.46372756919</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>87518.27456249634</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>106095.7874568847</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3305,6 +3635,21 @@
       <c r="AR10" t="n">
         <v>44061.0223603881</v>
       </c>
+      <c r="AS10" t="n">
+        <v>50589.30724076114</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>58224.22676166225</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>67179.34319592018</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>77713.66322612176</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>90141.9134188778</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3445,6 +3790,21 @@
       <c r="AR11" t="n">
         <v>-9726.557971457461</v>
       </c>
+      <c r="AS11" t="n">
+        <v>-14605.71379503702</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>-21464.00898133354</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>-31055.54257700904</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>-44409.51546444868</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>-62927.56157551002</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3584,6 +3944,21 @@
       </c>
       <c r="AR12" t="n">
         <v>-0.5102954804154141</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>-0.7090768402309638</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>-0.9642492908551845</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>-1.290998032100474</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>-1.70832487995135</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>-2.239975698570109</v>
       </c>
     </row>
     <row r="13">
@@ -3655,6 +4030,21 @@
       <c r="AR13" t="n">
         <v>399.440098842199</v>
       </c>
+      <c r="AS13" t="n">
+        <v>461.0689683546252</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>532.2064414558968</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>614.3195828987034</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>709.1018081262939</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>818.5078064992946</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3725,6 +4115,21 @@
       <c r="AR14" t="n">
         <v>195.2955612554993</v>
       </c>
+      <c r="AS14" t="n">
+        <v>217.6169705981405</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>242.4896172133479</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>270.2050961129335</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>301.0883303146256</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>335.5013800841112</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3795,6 +4200,21 @@
       <c r="AR15" t="n">
         <v>62.33879274111556</v>
       </c>
+      <c r="AS15" t="n">
+        <v>68.37323850649534</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>74.99182352279925</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>82.25109294392161</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>90.21306554057644</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>98.94576355085104</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3865,6 +4285,21 @@
       <c r="AR16" t="n">
         <v>0.6296847751627835</v>
       </c>
+      <c r="AS16" t="n">
+        <v>0.6906387727928824</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0.7574931668969624</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0.8308191206456731</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0.9112430862684492</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0.9994521570793038</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3935,6 +4370,21 @@
       <c r="AR17" t="n">
         <v>163.4017362536114</v>
       </c>
+      <c r="AS17" t="n">
+        <v>176.5829202327723</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>190.8273953070953</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>206.2209343445442</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>222.8562292824817</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>240.8334492706172</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4005,6 +4455,21 @@
       <c r="AR18" t="n">
         <v>811.329047770587</v>
       </c>
+      <c r="AS18" t="n">
+        <v>876.7768067203649</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>947.5040625195635</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>1023.936698153793</v>
+      </c>
+      <c r="AV18" t="n">
+        <v>1106.534951457735</v>
+      </c>
+      <c r="AW18" t="n">
+        <v>1195.796186429551</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4075,6 +4540,21 @@
       <c r="AR19" t="n">
         <v>1632.434921638175</v>
       </c>
+      <c r="AS19" t="n">
+        <v>1801.109543185191</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>1988.776833185599</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>2197.764223574542</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>2430.70562780798</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>2690.584037991505</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4145,6 +4625,21 @@
       <c r="AR20" t="n">
         <v>512.4389625106181</v>
       </c>
+      <c r="AS20" t="n">
+        <v>553.7760522980806</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>598.4476953047694</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>646.7228810804816</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>698.8922978474128</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>755.2700828744166</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4215,6 +4710,21 @@
       <c r="AR21" t="n">
         <v>276.3027743279826</v>
       </c>
+      <c r="AS21" t="n">
+        <v>298.5913851216713</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>322.6779589373413</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>348.7075326756021</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>376.8368429785384</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>407.2352700167731</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4285,6 +4795,21 @@
       <c r="AR22" t="n">
         <v>227.6142981295382</v>
       </c>
+      <c r="AS22" t="n">
+        <v>245.9753388915314</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>265.817516034824</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>287.2603088965867</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>310.4328348947174</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>335.4746270062092</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4355,6 +4880,21 @@
       <c r="AR23" t="n">
         <v>31.71577023203337</v>
       </c>
+      <c r="AS23" t="n">
+        <v>34.27419716221226</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>37.03900559626689</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>40.02684378185272</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>43.25570293653672</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>46.74502558161247</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4425,6 +4965,21 @@
       <c r="AR24" t="n">
         <v>21.26621488650494</v>
       </c>
+      <c r="AS24" t="n">
+        <v>22.9817039466966</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>24.83557695209633</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>26.83899696794059</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>29.00402755428327</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>31.34370540652035</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4493,6 +5048,21 @@
         <v>0</v>
       </c>
       <c r="AR25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4565,6 +5135,21 @@
       <c r="AR26" t="n">
         <v>1069.338020086677</v>
       </c>
+      <c r="AS26" t="n">
+        <v>1155.598677420192</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>1248.817752825298</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>1349.556563402464</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>1458.421706211489</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>1576.068710885532</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4635,6 +5220,21 @@
       <c r="AR27" t="n">
         <v>563.0969015514979</v>
       </c>
+      <c r="AS27" t="n">
+        <v>645.5108657649989</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>739.9590803603015</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>848.2076601720779</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>972.2839215964918</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>1114.515327105973</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4705,6 +5305,21 @@
       <c r="AR28" t="n">
         <v>0.0295423935929717</v>
       </c>
+      <c r="AS28" t="n">
+        <v>0.03133820171027384</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0.03324192694476528</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0.03526051484624112</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0.03740137212191884</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0.03967239768866034</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4775,6 +5390,21 @@
       <c r="AR29" t="n">
         <v>0</v>
       </c>
+      <c r="AS29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4845,6 +5475,21 @@
       <c r="AR30" t="n">
         <v>0</v>
       </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4985,6 +5630,21 @@
       <c r="AR31" t="n">
         <v>17165.83317641796</v>
       </c>
+      <c r="AS31" t="n">
+        <v>22757.84277724937</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>30171.5275076486</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>40000.3234513435</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>53030.98677408652</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>70306.57043696687</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5124,6 +5784,21 @@
       </c>
       <c r="AR32" t="n">
         <v>33935.8632174264</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>41415.72205011477</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>50544.22873945221</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>61684.76444222679</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>75280.80374729335</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>91873.56819926461</v>
       </c>
     </row>
     <row r="33">
@@ -5209,6 +5884,21 @@
       <c r="AR33" t="n">
         <v>8204.14004720465</v>
       </c>
+      <c r="AS33" t="n">
+        <v>11068.36563588981</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>14932.54834082069</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>20145.79272913773</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>27179.08259341841</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>36667.83137063861</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5293,6 +5983,21 @@
       <c r="AR34" t="n">
         <v>-6707.935324721199</v>
       </c>
+      <c r="AS34" t="n">
+        <v>-7795.869620019779</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>-9060.251804809008</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>-10529.69928534241</v>
+      </c>
+      <c r="AV34" t="n">
+        <v>-12237.47081520299</v>
+      </c>
+      <c r="AW34" t="n">
+        <v>-14222.21925762006</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5377,6 +6082,21 @@
       <c r="AR35" t="n">
         <v>25369.9732236226</v>
       </c>
+      <c r="AS35" t="n">
+        <v>33826.20841313917</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>45104.07584846929</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>60146.11618048123</v>
+      </c>
+      <c r="AV35" t="n">
+        <v>80210.06936750493</v>
+      </c>
+      <c r="AW35" t="n">
+        <v>106974.4018076055</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5461,6 +6181,21 @@
       <c r="AR36" t="n">
         <v>40643.7985421476</v>
       </c>
+      <c r="AS36" t="n">
+        <v>49211.59167013455</v>
+      </c>
+      <c r="AT36" t="n">
+        <v>59604.48054426122</v>
+      </c>
+      <c r="AU36" t="n">
+        <v>72214.46372756919</v>
+      </c>
+      <c r="AV36" t="n">
+        <v>87518.27456249634</v>
+      </c>
+      <c r="AW36" t="n">
+        <v>106095.7874568847</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5545,6 +6280,21 @@
       <c r="AR37" t="n">
         <v>-15273.82531852499</v>
       </c>
+      <c r="AS37" t="n">
+        <v>-15385.38325699538</v>
+      </c>
+      <c r="AT37" t="n">
+        <v>-14500.40469579193</v>
+      </c>
+      <c r="AU37" t="n">
+        <v>-12068.34754708797</v>
+      </c>
+      <c r="AV37" t="n">
+        <v>-7308.205194991409</v>
+      </c>
+      <c r="AW37" t="n">
+        <v>878.61435072081</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5629,6 +6379,21 @@
       <c r="AR38" t="n">
         <v>9672.667485852604</v>
       </c>
+      <c r="AS38" t="n">
+        <v>17410.80147453469</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>31339.44265416244</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>56410.99677749239</v>
+      </c>
+      <c r="AV38" t="n">
+        <v>101539.7941994863</v>
+      </c>
+      <c r="AW38" t="n">
+        <v>182771.6295590754</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5713,6 +6478,21 @@
       <c r="AR39" t="n">
         <v>4788.593570314097</v>
       </c>
+      <c r="AS39" t="n">
+        <v>4928.58974819982</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>5028.132764678535</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>5074.058878148728</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>5050.323659990036</v>
+      </c>
+      <c r="AW39" t="n">
+        <v>4937.441918850966</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5797,6 +6577,21 @@
       <c r="AR40" t="n">
         <v>-812.5642623582935</v>
       </c>
+      <c r="AS40" t="n">
+        <v>6954.007965739133</v>
+      </c>
+      <c r="AT40" t="n">
+        <v>21867.17072304905</v>
+      </c>
+      <c r="AU40" t="n">
+        <v>49416.70810855315</v>
+      </c>
+      <c r="AV40" t="n">
+        <v>99281.91266448495</v>
+      </c>
+      <c r="AW40" t="n">
+        <v>188587.6858286472</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5881,6 +6676,21 @@
       <c r="AR41" t="n">
         <v>-0.04263048365570885</v>
       </c>
+      <c r="AS41" t="n">
+        <v>0.3376025344932318</v>
+      </c>
+      <c r="AT41" t="n">
+        <v>0.9823609317833634</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>2.054282991927361</v>
+      </c>
+      <c r="AV41" t="n">
+        <v>3.819131097471031</v>
+      </c>
+      <c r="AW41" t="n">
+        <v>6.712985895676991</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5964,6 +6774,21 @@
       </c>
       <c r="AR42" t="n">
         <v>-0.8013280804545414</v>
+      </c>
+      <c r="AS42" t="n">
+        <v>-0.7469281610406228</v>
+      </c>
+      <c r="AT42" t="n">
+        <v>-0.6514162828197749</v>
+      </c>
+      <c r="AU42" t="n">
+        <v>-0.5016886404531684</v>
+      </c>
+      <c r="AV42" t="n">
+        <v>-0.2811286867650701</v>
+      </c>
+      <c r="AW42" t="n">
+        <v>0.03127524322816759</v>
       </c>
     </row>
     <row r="43">
@@ -6035,6 +6860,21 @@
       <c r="AR43" t="n">
         <v>2444.150752321788</v>
       </c>
+      <c r="AS43" t="n">
+        <v>2641.313900509854</v>
+      </c>
+      <c r="AT43" t="n">
+        <v>2854.381676089051</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>3084.637063099628</v>
+      </c>
+      <c r="AV43" t="n">
+        <v>3333.466540496054</v>
+      </c>
+      <c r="AW43" t="n">
+        <v>3602.36843080681</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6105,6 +6945,21 @@
       <c r="AR44" t="n">
         <v>2431.44304077439</v>
       </c>
+      <c r="AS44" t="n">
+        <v>2627.581091630563</v>
+      </c>
+      <c r="AT44" t="n">
+        <v>2839.541077999321</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>3068.599313386749</v>
+      </c>
+      <c r="AV44" t="n">
+        <v>3316.135068118876</v>
+      </c>
+      <c r="AW44" t="n">
+        <v>3583.638874594837</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6175,6 +7030,21 @@
       <c r="AR45" t="n">
         <v>665.0184356939575</v>
       </c>
+      <c r="AS45" t="n">
+        <v>718.6637062485543</v>
+      </c>
+      <c r="AT45" t="n">
+        <v>776.6363982675995</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>839.2855933446308</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>906.9885325579852</v>
+      </c>
+      <c r="AW45" t="n">
+        <v>980.15288802163</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6245,6 +7115,21 @@
       <c r="AR46" t="n">
         <v>1495.381818254201</v>
       </c>
+      <c r="AS46" t="n">
+        <v>1616.01029698045</v>
+      </c>
+      <c r="AT46" t="n">
+        <v>1746.369554630302</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>1887.244547289253</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>2039.48355136494</v>
+      </c>
+      <c r="AW46" t="n">
+        <v>2204.00327146932</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6315,6 +7200,21 @@
       <c r="AR47" t="n">
         <v>948.8040476303271</v>
       </c>
+      <c r="AS47" t="n">
+        <v>1025.34154960997</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>1108.053128548828</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>1197.436830833473</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>1294.030878929401</v>
+      </c>
+      <c r="AW47" t="n">
+        <v>1398.416912278583</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6385,6 +7285,21 @@
       <c r="AR48" t="n">
         <v>0.1282302625475281</v>
       </c>
+      <c r="AS48" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AT48" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AU48" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AV48" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="AW48" t="n">
+        <v>0.1282302625475281</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6455,6 +7370,21 @@
       <c r="AR49" t="n">
         <v>0.03488961903310435</v>
       </c>
+      <c r="AS49" t="n">
+        <v>0.03488961903310435</v>
+      </c>
+      <c r="AT49" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+      <c r="AU49" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+      <c r="AV49" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+      <c r="AW49" t="n">
+        <v>0.03488961903310435</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6467,7 +7397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI7"/>
+  <dimension ref="A1:AI12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7296,6 +8226,551 @@
         <v>0</v>
       </c>
       <c r="AI7" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.06160566932426947</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1142955282708081</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.1143413085694149</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.2415664077124058</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.6667517551006696</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.3257639488489026</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.220411627214698</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.3491195386969375</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.1621861634964107</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.02596506852221074</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.06862409785138872</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.428734058262854</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.09236232516636711</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.1765974049106775</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.04256567918702634</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.02688466848450283</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.01449598690303002</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0.01194158796506155</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0.00166394054862917</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0.00111571363415216</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.06160566932426947</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1142955282708081</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1143413085694149</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.2415664077124058</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.6667517551006696</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3257639488489026</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.220411627214698</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.3491195386969375</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.1621861634964107</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.02596506852221074</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.06862409785138872</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.428734058262854</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.09236232516636711</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.1765974049106775</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.04256567918702634</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.02688466848450283</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.01449598690303002</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.01194158796506155</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.00166394054862917</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0.00111571363415216</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.06160566932426947</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1142955282708081</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1143413085694149</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.2415664077124058</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.6667517551006696</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.3257639488489026</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.220411627214698</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.3491195386969375</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.1621861634964107</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.02596506852221074</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.06862409785138872</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.428734058262854</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.09236232516636711</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.1765974049106775</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.04256567918702634</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.02688466848450283</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.01449598690303002</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.01194158796506155</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.00166394054862917</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.00111571363415216</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.06160566932426947</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1142955282708081</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1143413085694149</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.2415664077124058</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.6667517551006696</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.3257639488489026</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.220411627214698</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.3491195386969375</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.1621861634964107</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.02596506852221074</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.06862409785138872</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.428734058262854</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.09236232516636711</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.1765974049106775</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.04256567918702634</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.02688466848450283</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.01449598690303002</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.01194158796506155</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.00166394054862917</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.00111571363415216</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.06160566932426947</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1142955282708081</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.1143413085694149</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.2415664077124058</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.6667517551006696</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.3257639488489026</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.220411627214698</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.3491195386969375</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.1621861634964107</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.02596506852221074</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.06862409785138872</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.428734058262854</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.09236232516636711</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.1765974049106775</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.04256567918702634</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.02688466848450283</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.01449598690303002</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0.01194158796506155</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.00166394054862917</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.00111571363415216</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI12" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
@@ -7312,7 +8787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9391,6 +10866,256 @@
         <v>0.08066734345284288</v>
       </c>
       <c r="P42" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B43" t="n">
+        <v>20598210188.72874</v>
+      </c>
+      <c r="C43" t="n">
+        <v>11430148300.89831</v>
+      </c>
+      <c r="D43" t="n">
+        <v>34045742595.36669</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1986448415.105047</v>
+      </c>
+      <c r="F43" t="n">
+        <v>14557116230.2894</v>
+      </c>
+      <c r="G43" t="n">
+        <v>33826208413.13918</v>
+      </c>
+      <c r="H43" t="n">
+        <v>49211591670.13455</v>
+      </c>
+      <c r="I43" t="n">
+        <v>226.8743734175154</v>
+      </c>
+      <c r="J43" t="n">
+        <v>36032191010.47174</v>
+      </c>
+      <c r="K43" t="n">
+        <v>50589307240.76114</v>
+      </c>
+      <c r="L43" t="n">
+        <v>35203923983.76576</v>
+      </c>
+      <c r="M43" t="n">
+        <v>-14605713795.03702</v>
+      </c>
+      <c r="N43" t="n">
+        <v>-0.7090768402309638</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B44" t="n">
+        <v>22259813084.53677</v>
+      </c>
+      <c r="C44" t="n">
+        <v>11849438448.04356</v>
+      </c>
+      <c r="D44" t="n">
+        <v>37937018730.67608</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2213581526.293798</v>
+      </c>
+      <c r="F44" t="n">
+        <v>18073626504.69237</v>
+      </c>
+      <c r="G44" t="n">
+        <v>45104075848.46929</v>
+      </c>
+      <c r="H44" t="n">
+        <v>59604480544.26122</v>
+      </c>
+      <c r="I44" t="n">
+        <v>240.8511210444257</v>
+      </c>
+      <c r="J44" t="n">
+        <v>40150600256.96988</v>
+      </c>
+      <c r="K44" t="n">
+        <v>58224226761.66225</v>
+      </c>
+      <c r="L44" t="n">
+        <v>43723822065.87031</v>
+      </c>
+      <c r="M44" t="n">
+        <v>-21464008981.33354</v>
+      </c>
+      <c r="N44" t="n">
+        <v>-0.9642492908551845</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B45" t="n">
+        <v>24055453071.82318</v>
+      </c>
+      <c r="C45" t="n">
+        <v>12284109342.91535</v>
+      </c>
+      <c r="D45" t="n">
+        <v>42273050327.51824</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2466685334.635314</v>
+      </c>
+      <c r="F45" t="n">
+        <v>22439607533.76663</v>
+      </c>
+      <c r="G45" t="n">
+        <v>60146116180.48123</v>
+      </c>
+      <c r="H45" t="n">
+        <v>72214463727.5692</v>
+      </c>
+      <c r="I45" t="n">
+        <v>255.6889155638682</v>
+      </c>
+      <c r="J45" t="n">
+        <v>44739735662.15356</v>
+      </c>
+      <c r="K45" t="n">
+        <v>67179343195.92019</v>
+      </c>
+      <c r="L45" t="n">
+        <v>55110995648.83223</v>
+      </c>
+      <c r="M45" t="n">
+        <v>-31055542577.00904</v>
+      </c>
+      <c r="N45" t="n">
+        <v>-1.290998032100474</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B46" t="n">
+        <v>25995942566.68169</v>
+      </c>
+      <c r="C46" t="n">
+        <v>12734725194.81419</v>
+      </c>
+      <c r="D46" t="n">
+        <v>47104670946.3204</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2748729363.626501</v>
+      </c>
+      <c r="F46" t="n">
+        <v>27860262916.17487</v>
+      </c>
+      <c r="G46" t="n">
+        <v>80210069367.50493</v>
+      </c>
+      <c r="H46" t="n">
+        <v>87518274562.49634</v>
+      </c>
+      <c r="I46" t="n">
+        <v>271.4408023459769</v>
+      </c>
+      <c r="J46" t="n">
+        <v>49853400309.9469</v>
+      </c>
+      <c r="K46" t="n">
+        <v>77713663226.12177</v>
+      </c>
+      <c r="L46" t="n">
+        <v>70405458031.13037</v>
+      </c>
+      <c r="M46" t="n">
+        <v>-44409515464.44868</v>
+      </c>
+      <c r="N46" t="n">
+        <v>-1.70832487995135</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0.03668282651348442</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B47" t="n">
+        <v>28092966194.08858</v>
+      </c>
+      <c r="C47" t="n">
+        <v>13201870909.83246</v>
+      </c>
+      <c r="D47" t="n">
+        <v>52488524196.15267</v>
+      </c>
+      <c r="E47" t="n">
+        <v>3063022675.96673</v>
+      </c>
+      <c r="F47" t="n">
+        <v>34590366546.75839</v>
+      </c>
+      <c r="G47" t="n">
+        <v>106974401807.6055</v>
+      </c>
+      <c r="H47" t="n">
+        <v>106095787456.8847</v>
+      </c>
+      <c r="I47" t="n">
+        <v>288.1630946564176</v>
+      </c>
+      <c r="J47" t="n">
+        <v>55551546872.1194</v>
+      </c>
+      <c r="K47" t="n">
+        <v>90141913418.87779</v>
+      </c>
+      <c r="L47" t="n">
+        <v>91020527769.5986</v>
+      </c>
+      <c r="M47" t="n">
+        <v>-62927561575.51003</v>
+      </c>
+      <c r="N47" t="n">
+        <v>-2.239975698570109</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0.08066734345284288</v>
+      </c>
+      <c r="P47" t="n">
         <v>0.03668282651348442</v>
       </c>
     </row>
@@ -9405,7 +11130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11061,6 +12786,286 @@
       </c>
       <c r="R42" t="n">
         <v>-812564262.3582935</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B43" t="n">
+        <v>22757842777.24937</v>
+      </c>
+      <c r="C43" t="n">
+        <v>41415722050.11477</v>
+      </c>
+      <c r="D43" t="n">
+        <v>11068365635.88981</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-7795869620.019779</v>
+      </c>
+      <c r="F43" t="n">
+        <v>29464893759.86501</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-12054092285.33032</v>
+      </c>
+      <c r="H43" t="n">
+        <v>9150975404.339296</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-4222385656.139477</v>
+      </c>
+      <c r="J43" t="n">
+        <v>33644.16979862229</v>
+      </c>
+      <c r="K43" t="n">
+        <v>329.9145258249793</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1956.748893081831</v>
+      </c>
+      <c r="M43" t="n">
+        <v>33826208413.13918</v>
+      </c>
+      <c r="N43" t="n">
+        <v>49211591670.13455</v>
+      </c>
+      <c r="O43" t="n">
+        <v>-15385383256.99538</v>
+      </c>
+      <c r="P43" t="n">
+        <v>17410801474.53469</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>4928589748.19982</v>
+      </c>
+      <c r="R43" t="n">
+        <v>6954007965.739134</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B44" t="n">
+        <v>30171527507.6486</v>
+      </c>
+      <c r="C44" t="n">
+        <v>50544228739.45222</v>
+      </c>
+      <c r="D44" t="n">
+        <v>14932548340.82069</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-9060251804.809008</v>
+      </c>
+      <c r="F44" t="n">
+        <v>53036808767.75702</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-21697366113.59458</v>
+      </c>
+      <c r="H44" t="n">
+        <v>9996180770.224312</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-4968048005.545777</v>
+      </c>
+      <c r="J44" t="n">
+        <v>34517.74297281641</v>
+      </c>
+      <c r="K44" t="n">
+        <v>352.5546125277872</v>
+      </c>
+      <c r="L44" t="n">
+        <v>2795.673787014151</v>
+      </c>
+      <c r="M44" t="n">
+        <v>45104075848.46929</v>
+      </c>
+      <c r="N44" t="n">
+        <v>59604480544.26122</v>
+      </c>
+      <c r="O44" t="n">
+        <v>-14500404695.79193</v>
+      </c>
+      <c r="P44" t="n">
+        <v>31339442654.16244</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>5028132764.678535</v>
+      </c>
+      <c r="R44" t="n">
+        <v>21867170723.04905</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B45" t="n">
+        <v>40000323451.3435</v>
+      </c>
+      <c r="C45" t="n">
+        <v>61684764442.22679</v>
+      </c>
+      <c r="D45" t="n">
+        <v>20145792729.13773</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-10529699285.34241</v>
+      </c>
+      <c r="F45" t="n">
+        <v>95466255781.96263</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-39055259004.47024</v>
+      </c>
+      <c r="H45" t="n">
+        <v>10919451268.94556</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-5845392390.796829</v>
+      </c>
+      <c r="J45" t="n">
+        <v>35413.99853433765</v>
+      </c>
+      <c r="K45" t="n">
+        <v>376.7483547558525</v>
+      </c>
+      <c r="L45" t="n">
+        <v>3994.27435529981</v>
+      </c>
+      <c r="M45" t="n">
+        <v>60146116180.48123</v>
+      </c>
+      <c r="N45" t="n">
+        <v>72214463727.5692</v>
+      </c>
+      <c r="O45" t="n">
+        <v>-12068347547.08797</v>
+      </c>
+      <c r="P45" t="n">
+        <v>56410996777.49239</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>5074058878.148727</v>
+      </c>
+      <c r="R45" t="n">
+        <v>49416708108.55315</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B46" t="n">
+        <v>53030986774.08652</v>
+      </c>
+      <c r="C46" t="n">
+        <v>75280803747.29335</v>
+      </c>
+      <c r="D46" t="n">
+        <v>27179082593.41841</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-12237470815.20299</v>
+      </c>
+      <c r="F46" t="n">
+        <v>171839260407.5327</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-70299466208.04643</v>
+      </c>
+      <c r="H46" t="n">
+        <v>11927997177.68621</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-6877673517.696171</v>
+      </c>
+      <c r="J46" t="n">
+        <v>36333.52543292721</v>
+      </c>
+      <c r="K46" t="n">
+        <v>402.6023707179679</v>
+      </c>
+      <c r="L46" t="n">
+        <v>5706.755809462743</v>
+      </c>
+      <c r="M46" t="n">
+        <v>80210069367.50493</v>
+      </c>
+      <c r="N46" t="n">
+        <v>87518274562.49634</v>
+      </c>
+      <c r="O46" t="n">
+        <v>-7308205194.991409</v>
+      </c>
+      <c r="P46" t="n">
+        <v>101539794199.4863</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>5050323659.990036</v>
+      </c>
+      <c r="R46" t="n">
+        <v>99281912664.48494</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B47" t="n">
+        <v>70306570436.96687</v>
+      </c>
+      <c r="C47" t="n">
+        <v>91873568199.26462</v>
+      </c>
+      <c r="D47" t="n">
+        <v>36667831370.63861</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-14222219257.62006</v>
+      </c>
+      <c r="F47" t="n">
+        <v>309310668733.559</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-126539039174.4836</v>
+      </c>
+      <c r="H47" t="n">
+        <v>13029694731.59517</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-8092252812.744205</v>
+      </c>
+      <c r="J47" t="n">
+        <v>37276.92791044665</v>
+      </c>
+      <c r="K47" t="n">
+        <v>430.2305952013188</v>
+      </c>
+      <c r="L47" t="n">
+        <v>8153.436387168824</v>
+      </c>
+      <c r="M47" t="n">
+        <v>106974401807.6055</v>
+      </c>
+      <c r="N47" t="n">
+        <v>106095787456.8847</v>
+      </c>
+      <c r="O47" t="n">
+        <v>878614350.7208099</v>
+      </c>
+      <c r="P47" t="n">
+        <v>182771629559.0754</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>4937441918.850965</v>
+      </c>
+      <c r="R47" t="n">
+        <v>188587685828.6472</v>
       </c>
     </row>
   </sheetData>
@@ -11074,7 +13079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11571,6 +13576,331 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B8" t="n">
+        <v>461068968.3546252</v>
+      </c>
+      <c r="C8" t="n">
+        <v>217616970.5981405</v>
+      </c>
+      <c r="D8" t="n">
+        <v>68373238.50649534</v>
+      </c>
+      <c r="E8" t="n">
+        <v>690638.7727928824</v>
+      </c>
+      <c r="F8" t="n">
+        <v>176582920.2327723</v>
+      </c>
+      <c r="G8" t="n">
+        <v>876776806.7203649</v>
+      </c>
+      <c r="H8" t="n">
+        <v>747749816.232054</v>
+      </c>
+      <c r="I8" t="n">
+        <v>924332736.4648263</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1801109543.185191</v>
+      </c>
+      <c r="K8" t="n">
+        <v>553776052.2980806</v>
+      </c>
+      <c r="L8" t="n">
+        <v>298591385.1216713</v>
+      </c>
+      <c r="M8" t="n">
+        <v>245975338.8915314</v>
+      </c>
+      <c r="N8" t="n">
+        <v>34274197.16221226</v>
+      </c>
+      <c r="O8" t="n">
+        <v>22981703.9466966</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1155598677.420192</v>
+      </c>
+      <c r="R8" t="n">
+        <v>645510865.7649989</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.03133820171027384</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B9" t="n">
+        <v>532206441.4558967</v>
+      </c>
+      <c r="C9" t="n">
+        <v>242489617.2133479</v>
+      </c>
+      <c r="D9" t="n">
+        <v>74991823.52279925</v>
+      </c>
+      <c r="E9" t="n">
+        <v>757493.1668969624</v>
+      </c>
+      <c r="F9" t="n">
+        <v>190827395.3070953</v>
+      </c>
+      <c r="G9" t="n">
+        <v>947504062.5195634</v>
+      </c>
+      <c r="H9" t="n">
+        <v>850445375.3589407</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1041272770.666036</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1988776833.185599</v>
+      </c>
+      <c r="K9" t="n">
+        <v>598447695.3047694</v>
+      </c>
+      <c r="L9" t="n">
+        <v>322677958.9373413</v>
+      </c>
+      <c r="M9" t="n">
+        <v>265817516.034824</v>
+      </c>
+      <c r="N9" t="n">
+        <v>37039005.59626689</v>
+      </c>
+      <c r="O9" t="n">
+        <v>24835576.95209633</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1248817752.825298</v>
+      </c>
+      <c r="R9" t="n">
+        <v>739959080.3603015</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.03324192694476528</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B10" t="n">
+        <v>614319582.8987035</v>
+      </c>
+      <c r="C10" t="n">
+        <v>270205096.1129335</v>
+      </c>
+      <c r="D10" t="n">
+        <v>82251092.94392161</v>
+      </c>
+      <c r="E10" t="n">
+        <v>830819.1206456731</v>
+      </c>
+      <c r="F10" t="n">
+        <v>206220934.3445442</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1023936698.153793</v>
+      </c>
+      <c r="H10" t="n">
+        <v>967606591.0762042</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1173827525.420748</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2197764223.574542</v>
+      </c>
+      <c r="K10" t="n">
+        <v>646722881.0804815</v>
+      </c>
+      <c r="L10" t="n">
+        <v>348707532.6756021</v>
+      </c>
+      <c r="M10" t="n">
+        <v>287260308.8965867</v>
+      </c>
+      <c r="N10" t="n">
+        <v>40026843.78185272</v>
+      </c>
+      <c r="O10" t="n">
+        <v>26838996.96794059</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1349556563.402464</v>
+      </c>
+      <c r="R10" t="n">
+        <v>848207660.1720779</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.03526051484624112</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B11" t="n">
+        <v>709101808.1262939</v>
+      </c>
+      <c r="C11" t="n">
+        <v>301088330.3146256</v>
+      </c>
+      <c r="D11" t="n">
+        <v>90213065.54057644</v>
+      </c>
+      <c r="E11" t="n">
+        <v>911243.0862684492</v>
+      </c>
+      <c r="F11" t="n">
+        <v>222856229.2824817</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1106534951.457735</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1101314447.067764</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1324170676.350246</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2430705627.807981</v>
+      </c>
+      <c r="K11" t="n">
+        <v>698892297.8474128</v>
+      </c>
+      <c r="L11" t="n">
+        <v>376836842.9785384</v>
+      </c>
+      <c r="M11" t="n">
+        <v>310432834.8947174</v>
+      </c>
+      <c r="N11" t="n">
+        <v>43255702.93653672</v>
+      </c>
+      <c r="O11" t="n">
+        <v>29004027.55428327</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1458421706.211489</v>
+      </c>
+      <c r="R11" t="n">
+        <v>972283921.5964918</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.03740137212191884</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B12" t="n">
+        <v>818507806.4992946</v>
+      </c>
+      <c r="C12" t="n">
+        <v>335501380.0841113</v>
+      </c>
+      <c r="D12" t="n">
+        <v>98945763.55085105</v>
+      </c>
+      <c r="E12" t="n">
+        <v>999452.1570793038</v>
+      </c>
+      <c r="F12" t="n">
+        <v>240833449.2706172</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1195796186.429551</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1253954402.291336</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1494787851.561954</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2690584037.991505</v>
+      </c>
+      <c r="K12" t="n">
+        <v>755270082.8744166</v>
+      </c>
+      <c r="L12" t="n">
+        <v>407235270.0167732</v>
+      </c>
+      <c r="M12" t="n">
+        <v>335474627.0062093</v>
+      </c>
+      <c r="N12" t="n">
+        <v>46745025.58161248</v>
+      </c>
+      <c r="O12" t="n">
+        <v>31343705.40652035</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1576068710.885532</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1114515327.105973</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.03967239768866034</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11585,7 +13915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11783,6 +14113,136 @@
         <v>0.1282302625475281</v>
       </c>
       <c r="H7" t="n">
+        <v>0.03488961903310435</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2641313900.509854</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2627581091.630563</v>
+      </c>
+      <c r="D8" t="n">
+        <v>718663706.2485542</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1616010296.980449</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1025341549.60997</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.03488961903310435</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2854381676.089051</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2839541077.999321</v>
+      </c>
+      <c r="D9" t="n">
+        <v>776636398.2675995</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1746369554.630302</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1108053128.548828</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3084637063.099628</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3068599313.386749</v>
+      </c>
+      <c r="D10" t="n">
+        <v>839285593.3446308</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1887244547.289253</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1197436830.833473</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3333466540.496054</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3316135068.118876</v>
+      </c>
+      <c r="D11" t="n">
+        <v>906988532.5579852</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2039483551.36494</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1294030878.929401</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.03488961903310436</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3602368430.80681</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3583638874.594837</v>
+      </c>
+      <c r="D12" t="n">
+        <v>980152888.02163</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2204003271.46932</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1398416912.278583</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.1282302625475281</v>
+      </c>
+      <c r="H12" t="n">
         <v>0.03488961903310435</v>
       </c>
     </row>
@@ -11797,7 +14257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13492,6 +15952,206 @@
         <v>0</v>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B43" t="n">
+        <v>20598210188.72874</v>
+      </c>
+      <c r="C43" t="n">
+        <v>36032191010.47174</v>
+      </c>
+      <c r="D43" t="n">
+        <v>14557116230.2894</v>
+      </c>
+      <c r="E43" t="n">
+        <v>33826208413.13918</v>
+      </c>
+      <c r="F43" t="n">
+        <v>49211591670.13455</v>
+      </c>
+      <c r="G43" t="n">
+        <v>35203923983.76576</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-14605713795.03702</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-0.7090768402309638</v>
+      </c>
+      <c r="J43" t="n">
+        <v>20598210188.72874</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B44" t="n">
+        <v>22259813084.53677</v>
+      </c>
+      <c r="C44" t="n">
+        <v>40150600256.96988</v>
+      </c>
+      <c r="D44" t="n">
+        <v>18073626504.69237</v>
+      </c>
+      <c r="E44" t="n">
+        <v>45104075848.46929</v>
+      </c>
+      <c r="F44" t="n">
+        <v>59604480544.26122</v>
+      </c>
+      <c r="G44" t="n">
+        <v>43723822065.87031</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-21464008981.33354</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-0.9642492908551845</v>
+      </c>
+      <c r="J44" t="n">
+        <v>22259813084.53677</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B45" t="n">
+        <v>24055453071.82318</v>
+      </c>
+      <c r="C45" t="n">
+        <v>44739735662.15356</v>
+      </c>
+      <c r="D45" t="n">
+        <v>22439607533.76663</v>
+      </c>
+      <c r="E45" t="n">
+        <v>60146116180.48123</v>
+      </c>
+      <c r="F45" t="n">
+        <v>72214463727.5692</v>
+      </c>
+      <c r="G45" t="n">
+        <v>55110995648.83223</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-31055542577.00904</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-1.290998032100474</v>
+      </c>
+      <c r="J45" t="n">
+        <v>24055453071.82318</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B46" t="n">
+        <v>25995942566.68169</v>
+      </c>
+      <c r="C46" t="n">
+        <v>49853400309.9469</v>
+      </c>
+      <c r="D46" t="n">
+        <v>27860262916.17487</v>
+      </c>
+      <c r="E46" t="n">
+        <v>80210069367.50493</v>
+      </c>
+      <c r="F46" t="n">
+        <v>87518274562.49634</v>
+      </c>
+      <c r="G46" t="n">
+        <v>70405458031.13037</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-44409515464.44868</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-1.70832487995135</v>
+      </c>
+      <c r="J46" t="n">
+        <v>25995942566.68169</v>
+      </c>
+      <c r="K46" t="n">
+        <v>-3.814697265625e-06</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B47" t="n">
+        <v>28092966194.08858</v>
+      </c>
+      <c r="C47" t="n">
+        <v>55551546872.1194</v>
+      </c>
+      <c r="D47" t="n">
+        <v>34590366546.75839</v>
+      </c>
+      <c r="E47" t="n">
+        <v>106974401807.6055</v>
+      </c>
+      <c r="F47" t="n">
+        <v>106095787456.8847</v>
+      </c>
+      <c r="G47" t="n">
+        <v>91020527769.5986</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-62927561575.51003</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-2.239975698570109</v>
+      </c>
+      <c r="J47" t="n">
+        <v>28092966194.08858</v>
+      </c>
+      <c r="K47" t="n">
+        <v>-3.814697265625e-06</v>
+      </c>
+      <c r="L47" t="inlineStr">
         <is>
           <t>WATCH</t>
         </is>
@@ -13508,7 +16168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP22"/>
+  <dimension ref="A1:AU22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13635,6 +16295,21 @@
       <c r="AP1" s="1" t="n">
         <v>2030</v>
       </c>
+      <c r="AQ1" s="1" t="n">
+        <v>2031</v>
+      </c>
+      <c r="AR1" s="1" t="n">
+        <v>2032</v>
+      </c>
+      <c r="AS1" s="1" t="n">
+        <v>2033</v>
+      </c>
+      <c r="AT1" s="1" t="n">
+        <v>2034</v>
+      </c>
+      <c r="AU1" s="1" t="n">
+        <v>2035</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -13765,6 +16440,21 @@
       <c r="AP2" t="n">
         <v>19060639070.40565</v>
       </c>
+      <c r="AQ2" t="n">
+        <v>20598210188.72874</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>22259813084.53677</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>24055453071.82318</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>25995942566.68169</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>28092966194.08858</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -13895,6 +16585,21 @@
       <c r="AP3" t="n">
         <v>32336223638.49695</v>
       </c>
+      <c r="AQ3" t="n">
+        <v>36032191010.47174</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>40150600256.96988</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>44739735662.15356</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>49853400309.9469</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>55551546872.1194</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -14025,6 +16730,21 @@
       <c r="AP4" t="n">
         <v>30553602461.45808</v>
       </c>
+      <c r="AQ4" t="n">
+        <v>34045742595.36669</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>37937018730.67608</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>42273050327.51824</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>47104670946.3204</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>52488524196.15267</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -14155,6 +16875,21 @@
       <c r="AP5" t="n">
         <v>1782621177.038872</v>
       </c>
+      <c r="AQ5" t="n">
+        <v>1986448415.105047</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>2213581526.293798</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>2466685334.635314</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>2748729363.626501</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>3063022675.96673</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -14285,6 +17020,21 @@
       <c r="AP6" t="n">
         <v>11724798721.89115</v>
       </c>
+      <c r="AQ6" t="n">
+        <v>14557116230.2894</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>18073626504.69237</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>22439607533.76663</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>27860262916.17487</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>34590366546.75839</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -14415,6 +17165,21 @@
       <c r="AP7" t="n">
         <v>11724798721.89115</v>
       </c>
+      <c r="AQ7" t="n">
+        <v>14557116230.2894</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>18073626504.69237</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>22439607533.76663</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>27860262916.17487</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>34590366546.75839</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -14545,6 +17310,21 @@
       <c r="AP8" t="n">
         <v>0</v>
       </c>
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -14675,6 +17455,21 @@
       <c r="AP9" t="n">
         <v>0</v>
       </c>
+      <c r="AQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -14805,6 +17600,21 @@
       <c r="AP10" t="n">
         <v>-15273825318.52499</v>
       </c>
+      <c r="AQ10" t="n">
+        <v>-15385383256.99538</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>-14500404695.79193</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>-12068347547.08797</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>-7308205194.991409</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>878614350.7208099</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -14935,6 +17745,21 @@
       <c r="AP11" t="n">
         <v>25369973223.6226</v>
       </c>
+      <c r="AQ11" t="n">
+        <v>33826208413.13918</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>45104075848.46929</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>60146116180.48123</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>80210069367.50493</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>106974401807.6055</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -15065,6 +17890,21 @@
       <c r="AP12" t="n">
         <v>40643798542.1476</v>
       </c>
+      <c r="AQ12" t="n">
+        <v>49211591670.13455</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>59604480544.26122</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>72214463727.5692</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>87518274562.49634</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>106095787456.8847</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -15194,6 +18034,21 @@
       </c>
       <c r="AP13" t="n">
         <v>-9726557971.457462</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>-14605713795.03702</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>-21464008981.33354</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>-31055542577.00904</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>-44409515464.44868</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>-62927561575.51003</v>
       </c>
     </row>
     <row r="14">
@@ -15269,6 +18124,21 @@
       <c r="AP14" t="n">
         <v>28733306556.25826</v>
       </c>
+      <c r="AQ14" t="n">
+        <v>38009011663.26343</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>53599255738.69921</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>80466449849.31558</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>127535736766.168</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>210864595753.164</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -15343,6 +18213,21 @@
       <c r="AP15" t="n">
         <v>33521900126.57235</v>
       </c>
+      <c r="AQ15" t="n">
+        <v>42937601411.46325</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>58627388503.37775</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>85540508727.46431</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>132586060426.158</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>215802037672.0149</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -15472,6 +18357,21 @@
       </c>
       <c r="AP16" t="n">
         <v>44061022360.3881</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>50589307240.76114</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>58224226761.66225</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>67179343195.92019</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>77713663226.12177</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>90141913418.87779</v>
       </c>
     </row>
     <row r="17">
@@ -15547,6 +18447,21 @@
       <c r="AP17" t="n">
         <v>1185676488.075397</v>
       </c>
+      <c r="AQ17" t="n">
+        <v>6905410400.991508</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>18476788246.40787</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>40800773065.31075</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>82732660116.21114</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>160250490799.8955</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -15676,6 +18591,21 @@
       </c>
       <c r="AP18" t="n">
         <v>11724798721.89115</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>14557116230.2894</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>18073626504.69237</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>22439607533.76663</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>27860262916.17487</v>
+      </c>
+      <c r="AU18" t="n">
+        <v>34590366546.75839</v>
       </c>
     </row>
     <row r="19">
@@ -15751,6 +18681,21 @@
       <c r="AP19" t="n">
         <v>-10539122233.81575</v>
       </c>
+      <c r="AQ19" t="n">
+        <v>-7651705829.297894</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>403161741.7154961</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>18361165531.54412</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>54872397200.03626</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>125660124253.1371</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -15825,6 +18770,21 @@
       <c r="AP20" t="n">
         <v>-812564262.3582935</v>
       </c>
+      <c r="AQ20" t="n">
+        <v>6954007965.739134</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>21867170723.04905</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>49416708108.55315</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>99281912664.48494</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>188587685828.6472</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -15899,6 +18859,21 @@
       <c r="AP21" t="n">
         <v>9672667485.852604</v>
       </c>
+      <c r="AQ21" t="n">
+        <v>17410801474.53469</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>31339442654.16244</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>56410996777.49239</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>101539794199.4863</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>182771629559.0754</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -15973,6 +18948,21 @@
       <c r="AP22" t="n">
         <v>4788593570.314096</v>
       </c>
+      <c r="AQ22" t="n">
+        <v>4928589748.19982</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>5028132764.678535</v>
+      </c>
+      <c r="AS22" t="n">
+        <v>5074058878.148727</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>5050323659.990036</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>4937441918.850965</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>